<commit_message>
PTLTR: ridge on the tendon cut, line on the ridge's slice (Mistovich 2018)
The lateral trochlear ridge is now taken on the tendon cut (the first slice
below the patella), or the nearest slice with a usable ridge, and PTLTR is
measured along the posterior condylar line drawn on that same slice, as in
Mistovich et al. 2018 (Fig. 2B). Previously the ridge was the most anterior
lateral point over the whole trochlea, against the knee's usual PBCL.

The usual PBCL is unchanged and still used by every other measurement;
pbcl.pbcl_on_slice draws the same bitangent on one given slice. ORS manual
agreement: ICC 0.73 (was 0.75), within noise; see VALIDATION.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Measurement methods.xlsx
+++ b/Measurement methods.xlsx
@@ -794,7 +794,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BONE. Ridge: femur BONE. Patella point: patella BONE. Reference direction (PBCL): femur BONE. Cartilage is used only to choose which slices are searched and to divide medial from lateral.</t>
+          <t>BONE. Ridge: femur BONE. Patella point: patella BONE. Reference line: femur BONE (the posterior condylar line on the ridge's slice). Cartilage is used only to choose which slices qualify and to divide medial from lateral.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Lateral trochlear ridge = the femur BONE point lateral of the sulcus with the greatest anterior projection beyond the PBCL. Patella point = the most lateral voxel of the patella BONE. Both are projected onto the PBCL direction (as for TT-TG); PTLTR is the distance between the projections.</t>
+          <t>On the tendon cut (the first axial slice below the patella BONE), or the nearest slice with a usable ridge: lateral trochlear ridge = the femur BONE point lateral of that slice's sulcus lying furthest anterior of the posterior condylar line drawn on the same slice. Patella point = the most lateral voxel of the patella BONE. Both are projected onto that line's direction (as for TT-TG); PTLTR is the distance between the projections.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>PBCL (bone); lateral trochlear ridge (bone); lateral patellar point (bone)</t>
+          <t>Posterior condylar line on the ridge's slice (bone; the knee's usual PBCL if that slice has no notch); lateral trochlear ridge (bone); lateral patellar point (bone)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>ICC 0.75 (n=43)</t>
+          <t>ICC 0.73 (n=43)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Adapted: the published PT-LTR measures from the patellar TENDON; this measures from the lateral edge of the patella BONE (no tendon label in the segmentation).</t>
+          <t>Adapted: ridge on the tendon cut and the line on the same slice, as in Mistovich 2018 (Fig. 2B); the published PT-LTR measures from the patellar TENDON, this from the lateral edge of the patella BONE (no tendon label in the segmentation), and along the posterior condylar line rather than along the tendon.</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr"/>
@@ -2010,7 +2010,7 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>KRA, TT-TG, sTT-TG, PTLTR, LTI, facet depths, trochlear depth</t>
+          <t>KRA, TT-TG, sTT-TG, LTI, facet depths, trochlear depth; PTLTR only when the ridge's slice has no notch (PTLTR otherwise draws the same bitangent on the ridge's slice)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -2215,7 +2215,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>BONE (femur). Cartilage only selects the slices searched and gives each slice's medial/lateral divide (its sulcus).</t>
+          <t>BONE (femur). Cartilage only decides which slices qualify and gives each slice's medial/lateral divide (its sulcus).</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>The femur BONE point lateral of each slice's own CARTILAGE sulcus with the greatest anterior projection beyond the PBCL, searched from the top of the trochlea to the condyle split, only on slices with a CARTILAGE sulcus of at least 2 mm.</t>
+          <t>On the tendon cut (the first axial slice below the patella BONE), or the nearest qualifying slice (a tie goes to the distal one): the femur BONE point lateral of the slice's own CARTILAGE sulcus lying furthest anterior of the posterior condylar line on that slice. A slice qualifies when it has a CARTILAGE sulcus of at least 2 mm and the condyles haven't split.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -2245,7 +2245,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>[Mistovich 2018] (lateral trochlear ridge). Detection: project-defined.</t>
+          <t>[Mistovich 2018] (ridge on the tendon cut, or the most visible cut). Detection: project-defined.</t>
         </is>
       </c>
     </row>
@@ -3047,22 +3047,22 @@
         <v>43</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>-2.4478</v>
+        <v>-2.7722</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>-12.5544</v>
+        <v>-13.0383</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>7.6588</v>
+        <v>7.4939</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>4.5709</v>
+        <v>4.7099</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>0.8054</v>
+        <v>0.7981</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>0.7477</v>
+        <v>0.7329</v>
       </c>
     </row>
     <row r="8">

</xml_diff>